<commit_message>
Change lupin in yr1 history from L to L1 (so that lupins and lupin fodder can be differentiated if they were the land use last year). No impact because no lf rotations hooked up atm.
</commit_message>
<xml_diff>
--- a/ExcelInputs/Rotation.xlsx
+++ b/ExcelInputs/Rotation.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1640" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1640" uniqueCount="188">
   <si>
     <t>AAAA2A1a</t>
   </si>
@@ -157,10 +157,10 @@
     <t>YYBNBl</t>
   </si>
   <si>
-    <t>YYNBLb</t>
-  </si>
-  <si>
-    <t>YYNBLbd</t>
+    <t>YYNBL1b</t>
+  </si>
+  <si>
+    <t>YYNBL1bd</t>
   </si>
   <si>
     <t>YYBLBz</t>
@@ -208,10 +208,10 @@
     <t>YYNWBl</t>
   </si>
   <si>
-    <t>YYWBLw</t>
-  </si>
-  <si>
-    <t>YYWBLwd</t>
+    <t>YYWBL1w</t>
+  </si>
+  <si>
+    <t>YYWBL1wd</t>
   </si>
   <si>
     <t>YYBLWb</t>
@@ -358,6 +358,9 @@
     <t>P</t>
   </si>
   <si>
+    <t>L1</t>
+  </si>
+  <si>
     <t>a</t>
   </si>
   <si>
@@ -511,7 +514,7 @@
     <t>YYBNB</t>
   </si>
   <si>
-    <t>YYNBL</t>
+    <t>YYNBL1</t>
   </si>
   <si>
     <t>YYBLB</t>
@@ -535,7 +538,7 @@
     <t>YYBNW</t>
   </si>
   <si>
-    <t>YYWBL</t>
+    <t>YYWBL1</t>
   </si>
   <si>
     <t>YYBLW</t>
@@ -958,7 +961,7 @@
         <v>106</v>
       </c>
       <c r="G1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="2" spans="1:7">
@@ -981,7 +984,7 @@
         <v>107</v>
       </c>
       <c r="G2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -1004,7 +1007,7 @@
         <v>108</v>
       </c>
       <c r="G3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1027,7 +1030,7 @@
         <v>96</v>
       </c>
       <c r="G4" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1050,7 +1053,7 @@
         <v>97</v>
       </c>
       <c r="G5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -1073,7 +1076,7 @@
         <v>109</v>
       </c>
       <c r="G6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -1096,7 +1099,7 @@
         <v>110</v>
       </c>
       <c r="G7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1119,7 +1122,7 @@
         <v>111</v>
       </c>
       <c r="G8" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1142,7 +1145,7 @@
         <v>97</v>
       </c>
       <c r="G9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1165,7 +1168,7 @@
         <v>109</v>
       </c>
       <c r="G10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1188,7 +1191,7 @@
         <v>112</v>
       </c>
       <c r="G11" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -1211,7 +1214,7 @@
         <v>110</v>
       </c>
       <c r="G12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -1234,7 +1237,7 @@
         <v>111</v>
       </c>
       <c r="G13" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1257,7 +1260,7 @@
         <v>94</v>
       </c>
       <c r="G14" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1280,7 +1283,7 @@
         <v>98</v>
       </c>
       <c r="G15" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1303,7 +1306,7 @@
         <v>98</v>
       </c>
       <c r="G16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -1326,7 +1329,7 @@
         <v>100</v>
       </c>
       <c r="G17" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -1349,7 +1352,7 @@
         <v>100</v>
       </c>
       <c r="G18" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -1372,7 +1375,7 @@
         <v>98</v>
       </c>
       <c r="G19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1395,7 +1398,7 @@
         <v>97</v>
       </c>
       <c r="G20" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1418,7 +1421,7 @@
         <v>97</v>
       </c>
       <c r="G21" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1441,7 +1444,7 @@
         <v>106</v>
       </c>
       <c r="G22" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1464,7 +1467,7 @@
         <v>106</v>
       </c>
       <c r="G23" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1487,7 +1490,7 @@
         <v>106</v>
       </c>
       <c r="G24" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1510,7 +1513,7 @@
         <v>99</v>
       </c>
       <c r="G25" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1533,7 +1536,7 @@
         <v>99</v>
       </c>
       <c r="G26" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1556,7 +1559,7 @@
         <v>99</v>
       </c>
       <c r="G27" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1579,7 +1582,7 @@
         <v>97</v>
       </c>
       <c r="G28" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1602,7 +1605,7 @@
         <v>97</v>
       </c>
       <c r="G29" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1625,7 +1628,7 @@
         <v>106</v>
       </c>
       <c r="G30" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1648,7 +1651,7 @@
         <v>106</v>
       </c>
       <c r="G31" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="32" spans="1:7">
@@ -1671,7 +1674,7 @@
         <v>106</v>
       </c>
       <c r="G32" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="33" spans="1:7">
@@ -1694,7 +1697,7 @@
         <v>106</v>
       </c>
       <c r="G33" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1717,7 +1720,7 @@
         <v>106</v>
       </c>
       <c r="G34" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="35" spans="1:7">
@@ -1740,7 +1743,7 @@
         <v>101</v>
       </c>
       <c r="G35" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="36" spans="1:7">
@@ -1763,7 +1766,7 @@
         <v>99</v>
       </c>
       <c r="G36" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1786,7 +1789,7 @@
         <v>106</v>
       </c>
       <c r="G37" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="38" spans="1:7">
@@ -1809,7 +1812,7 @@
         <v>110</v>
       </c>
       <c r="G38" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" spans="1:7">
@@ -1832,7 +1835,7 @@
         <v>106</v>
       </c>
       <c r="G39" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="40" spans="1:7">
@@ -1855,7 +1858,7 @@
         <v>97</v>
       </c>
       <c r="G40" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="41" spans="1:7">
@@ -1878,7 +1881,7 @@
         <v>97</v>
       </c>
       <c r="G41" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="42" spans="1:7">
@@ -1901,7 +1904,7 @@
         <v>99</v>
       </c>
       <c r="G42" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="43" spans="1:7">
@@ -1924,7 +1927,7 @@
         <v>99</v>
       </c>
       <c r="G43" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -1947,7 +1950,7 @@
         <v>99</v>
       </c>
       <c r="G44" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="45" spans="1:7">
@@ -1970,7 +1973,7 @@
         <v>99</v>
       </c>
       <c r="G45" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="46" spans="1:7">
@@ -1993,7 +1996,7 @@
         <v>99</v>
       </c>
       <c r="G46" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="47" spans="1:7">
@@ -2013,10 +2016,10 @@
         <v>99</v>
       </c>
       <c r="F47" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="G47" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="48" spans="1:7">
@@ -2036,10 +2039,10 @@
         <v>99</v>
       </c>
       <c r="F48" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="G48" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="49" spans="1:7">
@@ -2062,7 +2065,7 @@
         <v>99</v>
       </c>
       <c r="G49" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="50" spans="1:7">
@@ -2085,7 +2088,7 @@
         <v>99</v>
       </c>
       <c r="G50" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="51" spans="1:7">
@@ -2108,7 +2111,7 @@
         <v>97</v>
       </c>
       <c r="G51" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -2131,7 +2134,7 @@
         <v>97</v>
       </c>
       <c r="G52" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -2154,7 +2157,7 @@
         <v>97</v>
       </c>
       <c r="G53" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="54" spans="1:7">
@@ -2177,7 +2180,7 @@
         <v>97</v>
       </c>
       <c r="G54" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="55" spans="1:7">
@@ -2200,7 +2203,7 @@
         <v>98</v>
       </c>
       <c r="G55" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="56" spans="1:7">
@@ -2223,7 +2226,7 @@
         <v>98</v>
       </c>
       <c r="G56" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="57" spans="1:7">
@@ -2246,7 +2249,7 @@
         <v>99</v>
       </c>
       <c r="G57" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="58" spans="1:7">
@@ -2269,7 +2272,7 @@
         <v>99</v>
       </c>
       <c r="G58" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="59" spans="1:7">
@@ -2292,7 +2295,7 @@
         <v>97</v>
       </c>
       <c r="G59" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="60" spans="1:7">
@@ -2315,7 +2318,7 @@
         <v>97</v>
       </c>
       <c r="G60" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="61" spans="1:7">
@@ -2338,7 +2341,7 @@
         <v>98</v>
       </c>
       <c r="G61" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="62" spans="1:7">
@@ -2361,7 +2364,7 @@
         <v>98</v>
       </c>
       <c r="G62" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="63" spans="1:7">
@@ -2384,7 +2387,7 @@
         <v>99</v>
       </c>
       <c r="G63" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="64" spans="1:7">
@@ -2404,10 +2407,10 @@
         <v>99</v>
       </c>
       <c r="F64" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="G64" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="65" spans="1:7">
@@ -2427,10 +2430,10 @@
         <v>99</v>
       </c>
       <c r="F65" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
       <c r="G65" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="66" spans="1:7">
@@ -2453,7 +2456,7 @@
         <v>98</v>
       </c>
       <c r="G66" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -2476,7 +2479,7 @@
         <v>98</v>
       </c>
       <c r="G67" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -2499,7 +2502,7 @@
         <v>99</v>
       </c>
       <c r="G68" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="69" spans="1:7">
@@ -2522,7 +2525,7 @@
         <v>99</v>
       </c>
       <c r="G69" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="70" spans="1:7">
@@ -2545,7 +2548,7 @@
         <v>97</v>
       </c>
       <c r="G70" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="71" spans="1:7">
@@ -2568,7 +2571,7 @@
         <v>97</v>
       </c>
       <c r="G71" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -2591,7 +2594,7 @@
         <v>98</v>
       </c>
       <c r="G72" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -2614,7 +2617,7 @@
         <v>98</v>
       </c>
       <c r="G73" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="74" spans="1:7">
@@ -2637,7 +2640,7 @@
         <v>99</v>
       </c>
       <c r="G74" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="75" spans="1:7">
@@ -2660,7 +2663,7 @@
         <v>106</v>
       </c>
       <c r="G75" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="76" spans="1:7">
@@ -2683,7 +2686,7 @@
         <v>98</v>
       </c>
       <c r="G76" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="77" spans="1:7">
@@ -2706,7 +2709,7 @@
         <v>98</v>
       </c>
       <c r="G77" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="78" spans="1:7">
@@ -2729,7 +2732,7 @@
         <v>97</v>
       </c>
       <c r="G78" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="79" spans="1:7">
@@ -2752,7 +2755,7 @@
         <v>97</v>
       </c>
       <c r="G79" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="80" spans="1:7">
@@ -2775,7 +2778,7 @@
         <v>96</v>
       </c>
       <c r="G80" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="81" spans="1:7">
@@ -2798,7 +2801,7 @@
         <v>96</v>
       </c>
       <c r="G81" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="82" spans="1:7">
@@ -2821,7 +2824,7 @@
         <v>96</v>
       </c>
       <c r="G82" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="83" spans="1:7">
@@ -2844,7 +2847,7 @@
         <v>96</v>
       </c>
       <c r="G83" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="84" spans="1:7">
@@ -2867,7 +2870,7 @@
         <v>96</v>
       </c>
       <c r="G84" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="85" spans="1:7">
@@ -2890,7 +2893,7 @@
         <v>99</v>
       </c>
       <c r="G85" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="86" spans="1:7">
@@ -2913,7 +2916,7 @@
         <v>99</v>
       </c>
       <c r="G86" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="87" spans="1:7">
@@ -2936,7 +2939,7 @@
         <v>99</v>
       </c>
       <c r="G87" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="88" spans="1:7">
@@ -2959,7 +2962,7 @@
         <v>98</v>
       </c>
       <c r="G88" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="89" spans="1:7">
@@ -2982,7 +2985,7 @@
         <v>100</v>
       </c>
       <c r="G89" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="90" spans="1:7">
@@ -3005,7 +3008,7 @@
         <v>100</v>
       </c>
       <c r="G90" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="91" spans="1:7">
@@ -3028,7 +3031,7 @@
         <v>98</v>
       </c>
       <c r="G91" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="92" spans="1:7">
@@ -3051,7 +3054,7 @@
         <v>98</v>
       </c>
       <c r="G92" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>
@@ -3069,7 +3072,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C1">
         <v>1</v>
@@ -3080,7 +3083,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -3091,7 +3094,7 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -3102,7 +3105,7 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -3113,7 +3116,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -3124,7 +3127,7 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -3135,7 +3138,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C7">
         <v>1</v>
@@ -3146,7 +3149,7 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -3157,7 +3160,7 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -3168,7 +3171,7 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -3179,7 +3182,7 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -3190,7 +3193,7 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C12">
         <v>1</v>
@@ -3201,7 +3204,7 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C13">
         <v>1</v>
@@ -3212,7 +3215,7 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -3223,7 +3226,7 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -3234,7 +3237,7 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C16">
         <v>1</v>
@@ -3245,7 +3248,7 @@
         <v>14</v>
       </c>
       <c r="B17" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -3256,7 +3259,7 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -3267,7 +3270,7 @@
         <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -3278,7 +3281,7 @@
         <v>16</v>
       </c>
       <c r="B20" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -3289,7 +3292,7 @@
         <v>16</v>
       </c>
       <c r="B21" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -3300,7 +3303,7 @@
         <v>17</v>
       </c>
       <c r="B22" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -3311,7 +3314,7 @@
         <v>17</v>
       </c>
       <c r="B23" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -3322,7 +3325,7 @@
         <v>18</v>
       </c>
       <c r="B24" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -3333,7 +3336,7 @@
         <v>18</v>
       </c>
       <c r="B25" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C25">
         <v>1</v>
@@ -3344,7 +3347,7 @@
         <v>19</v>
       </c>
       <c r="B26" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -3355,7 +3358,7 @@
         <v>19</v>
       </c>
       <c r="B27" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -3366,7 +3369,7 @@
         <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -3377,7 +3380,7 @@
         <v>20</v>
       </c>
       <c r="B29" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -3388,7 +3391,7 @@
         <v>21</v>
       </c>
       <c r="B30" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -3399,7 +3402,7 @@
         <v>21</v>
       </c>
       <c r="B31" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -3410,7 +3413,7 @@
         <v>22</v>
       </c>
       <c r="B32" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -3421,7 +3424,7 @@
         <v>22</v>
       </c>
       <c r="B33" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -3432,7 +3435,7 @@
         <v>23</v>
       </c>
       <c r="B34" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -3443,7 +3446,7 @@
         <v>23</v>
       </c>
       <c r="B35" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -3454,7 +3457,7 @@
         <v>24</v>
       </c>
       <c r="B36" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -3465,7 +3468,7 @@
         <v>24</v>
       </c>
       <c r="B37" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -3476,7 +3479,7 @@
         <v>25</v>
       </c>
       <c r="B38" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -3487,7 +3490,7 @@
         <v>25</v>
       </c>
       <c r="B39" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C39">
         <v>1</v>
@@ -3498,7 +3501,7 @@
         <v>26</v>
       </c>
       <c r="B40" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C40">
         <v>1</v>
@@ -3509,7 +3512,7 @@
         <v>26</v>
       </c>
       <c r="B41" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -3520,7 +3523,7 @@
         <v>27</v>
       </c>
       <c r="B42" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C42">
         <v>1</v>
@@ -3531,7 +3534,7 @@
         <v>27</v>
       </c>
       <c r="B43" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -3542,7 +3545,7 @@
         <v>28</v>
       </c>
       <c r="B44" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C44">
         <v>1</v>
@@ -3553,7 +3556,7 @@
         <v>28</v>
       </c>
       <c r="B45" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -3564,7 +3567,7 @@
         <v>29</v>
       </c>
       <c r="B46" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -3575,7 +3578,7 @@
         <v>29</v>
       </c>
       <c r="B47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -3586,7 +3589,7 @@
         <v>30</v>
       </c>
       <c r="B48" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -3597,7 +3600,7 @@
         <v>30</v>
       </c>
       <c r="B49" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -3608,7 +3611,7 @@
         <v>31</v>
       </c>
       <c r="B50" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -3619,7 +3622,7 @@
         <v>31</v>
       </c>
       <c r="B51" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -3630,7 +3633,7 @@
         <v>32</v>
       </c>
       <c r="B52" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -3641,7 +3644,7 @@
         <v>32</v>
       </c>
       <c r="B53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -3652,7 +3655,7 @@
         <v>33</v>
       </c>
       <c r="B54" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -3663,7 +3666,7 @@
         <v>33</v>
       </c>
       <c r="B55" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C55">
         <v>1</v>
@@ -3674,7 +3677,7 @@
         <v>34</v>
       </c>
       <c r="B56" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -3685,7 +3688,7 @@
         <v>34</v>
       </c>
       <c r="B57" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C57">
         <v>1</v>
@@ -3696,7 +3699,7 @@
         <v>35</v>
       </c>
       <c r="B58" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C58">
         <v>1</v>
@@ -3707,7 +3710,7 @@
         <v>35</v>
       </c>
       <c r="B59" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -3718,7 +3721,7 @@
         <v>36</v>
       </c>
       <c r="B60" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C60">
         <v>1</v>
@@ -3729,7 +3732,7 @@
         <v>36</v>
       </c>
       <c r="B61" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C61">
         <v>1</v>
@@ -3740,7 +3743,7 @@
         <v>37</v>
       </c>
       <c r="B62" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C62">
         <v>1</v>
@@ -3751,7 +3754,7 @@
         <v>37</v>
       </c>
       <c r="B63" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C63">
         <v>1</v>
@@ -3762,7 +3765,7 @@
         <v>38</v>
       </c>
       <c r="B64" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C64">
         <v>1</v>
@@ -3773,7 +3776,7 @@
         <v>38</v>
       </c>
       <c r="B65" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C65">
         <v>1</v>
@@ -3784,7 +3787,7 @@
         <v>39</v>
       </c>
       <c r="B66" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C66">
         <v>1</v>
@@ -3795,7 +3798,7 @@
         <v>39</v>
       </c>
       <c r="B67" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C67">
         <v>1</v>
@@ -3806,7 +3809,7 @@
         <v>40</v>
       </c>
       <c r="B68" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C68">
         <v>1</v>
@@ -3817,7 +3820,7 @@
         <v>40</v>
       </c>
       <c r="B69" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C69">
         <v>1</v>
@@ -3828,7 +3831,7 @@
         <v>41</v>
       </c>
       <c r="B70" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C70">
         <v>1</v>
@@ -3839,7 +3842,7 @@
         <v>41</v>
       </c>
       <c r="B71" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -3850,7 +3853,7 @@
         <v>42</v>
       </c>
       <c r="B72" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C72">
         <v>1</v>
@@ -3861,7 +3864,7 @@
         <v>42</v>
       </c>
       <c r="B73" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C73">
         <v>1</v>
@@ -3872,7 +3875,7 @@
         <v>43</v>
       </c>
       <c r="B74" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C74">
         <v>1</v>
@@ -3883,7 +3886,7 @@
         <v>43</v>
       </c>
       <c r="B75" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C75">
         <v>1</v>
@@ -3894,7 +3897,7 @@
         <v>44</v>
       </c>
       <c r="B76" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C76">
         <v>1</v>
@@ -3905,7 +3908,7 @@
         <v>44</v>
       </c>
       <c r="B77" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C77">
         <v>1</v>
@@ -3916,7 +3919,7 @@
         <v>45</v>
       </c>
       <c r="B78" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C78">
         <v>1</v>
@@ -3927,7 +3930,7 @@
         <v>45</v>
       </c>
       <c r="B79" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C79">
         <v>1</v>
@@ -3938,7 +3941,7 @@
         <v>46</v>
       </c>
       <c r="B80" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C80">
         <v>1</v>
@@ -3949,7 +3952,7 @@
         <v>46</v>
       </c>
       <c r="B81" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C81">
         <v>1</v>
@@ -3960,7 +3963,7 @@
         <v>47</v>
       </c>
       <c r="B82" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C82">
         <v>1</v>
@@ -3971,7 +3974,7 @@
         <v>47</v>
       </c>
       <c r="B83" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C83">
         <v>1</v>
@@ -3982,7 +3985,7 @@
         <v>48</v>
       </c>
       <c r="B84" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C84">
         <v>1</v>
@@ -3993,7 +3996,7 @@
         <v>48</v>
       </c>
       <c r="B85" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C85">
         <v>1</v>
@@ -4004,7 +4007,7 @@
         <v>49</v>
       </c>
       <c r="B86" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C86">
         <v>1</v>
@@ -4015,7 +4018,7 @@
         <v>49</v>
       </c>
       <c r="B87" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C87">
         <v>1</v>
@@ -4026,7 +4029,7 @@
         <v>50</v>
       </c>
       <c r="B88" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C88">
         <v>1</v>
@@ -4037,7 +4040,7 @@
         <v>50</v>
       </c>
       <c r="B89" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C89">
         <v>1</v>
@@ -4048,7 +4051,7 @@
         <v>51</v>
       </c>
       <c r="B90" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C90">
         <v>1</v>
@@ -4059,7 +4062,7 @@
         <v>51</v>
       </c>
       <c r="B91" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C91">
         <v>1</v>
@@ -4070,7 +4073,7 @@
         <v>52</v>
       </c>
       <c r="B92" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C92">
         <v>1</v>
@@ -4081,7 +4084,7 @@
         <v>52</v>
       </c>
       <c r="B93" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C93">
         <v>1</v>
@@ -4092,7 +4095,7 @@
         <v>53</v>
       </c>
       <c r="B94" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C94">
         <v>1</v>
@@ -4103,7 +4106,7 @@
         <v>53</v>
       </c>
       <c r="B95" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C95">
         <v>1</v>
@@ -4114,7 +4117,7 @@
         <v>54</v>
       </c>
       <c r="B96" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C96">
         <v>1</v>
@@ -4125,7 +4128,7 @@
         <v>54</v>
       </c>
       <c r="B97" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C97">
         <v>1</v>
@@ -4136,7 +4139,7 @@
         <v>55</v>
       </c>
       <c r="B98" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C98">
         <v>1</v>
@@ -4147,7 +4150,7 @@
         <v>55</v>
       </c>
       <c r="B99" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C99">
         <v>1</v>
@@ -4158,7 +4161,7 @@
         <v>56</v>
       </c>
       <c r="B100" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C100">
         <v>1</v>
@@ -4169,7 +4172,7 @@
         <v>56</v>
       </c>
       <c r="B101" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C101">
         <v>1</v>
@@ -4180,7 +4183,7 @@
         <v>57</v>
       </c>
       <c r="B102" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C102">
         <v>1</v>
@@ -4191,7 +4194,7 @@
         <v>57</v>
       </c>
       <c r="B103" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C103">
         <v>1</v>
@@ -4202,7 +4205,7 @@
         <v>58</v>
       </c>
       <c r="B104" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C104">
         <v>1</v>
@@ -4213,7 +4216,7 @@
         <v>58</v>
       </c>
       <c r="B105" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C105">
         <v>1</v>
@@ -4224,7 +4227,7 @@
         <v>59</v>
       </c>
       <c r="B106" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C106">
         <v>1</v>
@@ -4235,7 +4238,7 @@
         <v>59</v>
       </c>
       <c r="B107" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C107">
         <v>1</v>
@@ -4246,7 +4249,7 @@
         <v>60</v>
       </c>
       <c r="B108" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C108">
         <v>1</v>
@@ -4257,7 +4260,7 @@
         <v>60</v>
       </c>
       <c r="B109" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C109">
         <v>1</v>
@@ -4268,7 +4271,7 @@
         <v>61</v>
       </c>
       <c r="B110" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C110">
         <v>1</v>
@@ -4279,7 +4282,7 @@
         <v>61</v>
       </c>
       <c r="B111" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C111">
         <v>1</v>
@@ -4290,7 +4293,7 @@
         <v>62</v>
       </c>
       <c r="B112" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C112">
         <v>1</v>
@@ -4301,7 +4304,7 @@
         <v>62</v>
       </c>
       <c r="B113" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C113">
         <v>1</v>
@@ -4312,7 +4315,7 @@
         <v>63</v>
       </c>
       <c r="B114" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C114">
         <v>1</v>
@@ -4323,7 +4326,7 @@
         <v>63</v>
       </c>
       <c r="B115" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C115">
         <v>1</v>
@@ -4334,7 +4337,7 @@
         <v>64</v>
       </c>
       <c r="B116" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C116">
         <v>1</v>
@@ -4345,7 +4348,7 @@
         <v>64</v>
       </c>
       <c r="B117" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C117">
         <v>1</v>
@@ -4356,7 +4359,7 @@
         <v>65</v>
       </c>
       <c r="B118" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C118">
         <v>1</v>
@@ -4367,7 +4370,7 @@
         <v>65</v>
       </c>
       <c r="B119" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C119">
         <v>1</v>
@@ -4378,7 +4381,7 @@
         <v>66</v>
       </c>
       <c r="B120" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C120">
         <v>1</v>
@@ -4389,7 +4392,7 @@
         <v>66</v>
       </c>
       <c r="B121" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C121">
         <v>1</v>
@@ -4400,7 +4403,7 @@
         <v>67</v>
       </c>
       <c r="B122" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C122">
         <v>1</v>
@@ -4411,7 +4414,7 @@
         <v>67</v>
       </c>
       <c r="B123" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C123">
         <v>1</v>
@@ -4422,7 +4425,7 @@
         <v>68</v>
       </c>
       <c r="B124" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C124">
         <v>1</v>
@@ -4433,7 +4436,7 @@
         <v>68</v>
       </c>
       <c r="B125" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C125">
         <v>1</v>
@@ -4444,7 +4447,7 @@
         <v>69</v>
       </c>
       <c r="B126" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C126">
         <v>1</v>
@@ -4455,7 +4458,7 @@
         <v>69</v>
       </c>
       <c r="B127" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C127">
         <v>1</v>
@@ -4466,7 +4469,7 @@
         <v>70</v>
       </c>
       <c r="B128" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C128">
         <v>1</v>
@@ -4477,7 +4480,7 @@
         <v>70</v>
       </c>
       <c r="B129" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C129">
         <v>1</v>
@@ -4488,7 +4491,7 @@
         <v>71</v>
       </c>
       <c r="B130" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C130">
         <v>1</v>
@@ -4499,7 +4502,7 @@
         <v>71</v>
       </c>
       <c r="B131" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C131">
         <v>1</v>
@@ -4510,7 +4513,7 @@
         <v>72</v>
       </c>
       <c r="B132" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C132">
         <v>1</v>
@@ -4521,7 +4524,7 @@
         <v>72</v>
       </c>
       <c r="B133" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C133">
         <v>1</v>
@@ -4532,7 +4535,7 @@
         <v>73</v>
       </c>
       <c r="B134" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C134">
         <v>1</v>
@@ -4543,7 +4546,7 @@
         <v>73</v>
       </c>
       <c r="B135" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C135">
         <v>1</v>
@@ -4554,7 +4557,7 @@
         <v>74</v>
       </c>
       <c r="B136" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C136">
         <v>1</v>
@@ -4565,7 +4568,7 @@
         <v>74</v>
       </c>
       <c r="B137" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C137">
         <v>1</v>
@@ -4576,7 +4579,7 @@
         <v>75</v>
       </c>
       <c r="B138" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C138">
         <v>1</v>
@@ -4587,7 +4590,7 @@
         <v>75</v>
       </c>
       <c r="B139" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C139">
         <v>1</v>
@@ -4598,7 +4601,7 @@
         <v>76</v>
       </c>
       <c r="B140" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C140">
         <v>1</v>
@@ -4609,7 +4612,7 @@
         <v>76</v>
       </c>
       <c r="B141" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C141">
         <v>1</v>
@@ -4620,7 +4623,7 @@
         <v>77</v>
       </c>
       <c r="B142" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C142">
         <v>1</v>
@@ -4631,7 +4634,7 @@
         <v>78</v>
       </c>
       <c r="B143" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C143">
         <v>1</v>
@@ -4642,7 +4645,7 @@
         <v>79</v>
       </c>
       <c r="B144" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C144">
         <v>1</v>
@@ -4653,7 +4656,7 @@
         <v>79</v>
       </c>
       <c r="B145" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C145">
         <v>1</v>
@@ -4664,7 +4667,7 @@
         <v>80</v>
       </c>
       <c r="B146" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C146">
         <v>1</v>
@@ -4675,7 +4678,7 @@
         <v>80</v>
       </c>
       <c r="B147" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C147">
         <v>1</v>
@@ -4686,7 +4689,7 @@
         <v>81</v>
       </c>
       <c r="B148" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C148">
         <v>1</v>
@@ -4697,7 +4700,7 @@
         <v>81</v>
       </c>
       <c r="B149" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C149">
         <v>1</v>
@@ -4708,7 +4711,7 @@
         <v>82</v>
       </c>
       <c r="B150" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C150">
         <v>1</v>
@@ -4719,7 +4722,7 @@
         <v>82</v>
       </c>
       <c r="B151" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C151">
         <v>1</v>
@@ -4730,7 +4733,7 @@
         <v>83</v>
       </c>
       <c r="B152" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C152">
         <v>1</v>
@@ -4741,7 +4744,7 @@
         <v>83</v>
       </c>
       <c r="B153" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C153">
         <v>1</v>
@@ -4752,7 +4755,7 @@
         <v>84</v>
       </c>
       <c r="B154" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C154">
         <v>1</v>
@@ -4763,7 +4766,7 @@
         <v>84</v>
       </c>
       <c r="B155" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C155">
         <v>1</v>
@@ -4774,7 +4777,7 @@
         <v>85</v>
       </c>
       <c r="B156" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C156">
         <v>1</v>
@@ -4785,7 +4788,7 @@
         <v>85</v>
       </c>
       <c r="B157" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C157">
         <v>1</v>
@@ -4796,7 +4799,7 @@
         <v>86</v>
       </c>
       <c r="B158" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C158">
         <v>1</v>
@@ -4807,7 +4810,7 @@
         <v>86</v>
       </c>
       <c r="B159" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C159">
         <v>1</v>
@@ -4818,7 +4821,7 @@
         <v>87</v>
       </c>
       <c r="B160" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C160">
         <v>1</v>
@@ -4829,7 +4832,7 @@
         <v>87</v>
       </c>
       <c r="B161" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C161">
         <v>1</v>
@@ -4840,7 +4843,7 @@
         <v>88</v>
       </c>
       <c r="B162" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C162">
         <v>1</v>
@@ -4851,7 +4854,7 @@
         <v>88</v>
       </c>
       <c r="B163" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C163">
         <v>1</v>
@@ -4862,7 +4865,7 @@
         <v>89</v>
       </c>
       <c r="B164" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C164">
         <v>1</v>
@@ -4873,7 +4876,7 @@
         <v>89</v>
       </c>
       <c r="B165" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C165">
         <v>1</v>
@@ -4884,7 +4887,7 @@
         <v>90</v>
       </c>
       <c r="B166" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C166">
         <v>1</v>
@@ -4895,7 +4898,7 @@
         <v>90</v>
       </c>
       <c r="B167" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C167">
         <v>1</v>
@@ -4906,7 +4909,7 @@
         <v>91</v>
       </c>
       <c r="B168" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C168">
         <v>1</v>
@@ -4917,7 +4920,7 @@
         <v>91</v>
       </c>
       <c r="B169" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C169">
         <v>1</v>
@@ -4938,7 +4941,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C1">
         <v>-1</v>
@@ -4949,7 +4952,7 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C2">
         <v>-1</v>
@@ -4960,7 +4963,7 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C3">
         <v>-1</v>
@@ -4971,7 +4974,7 @@
         <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C4">
         <v>-1</v>
@@ -4982,7 +4985,7 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C5">
         <v>-1</v>
@@ -4993,7 +4996,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C6">
         <v>-1</v>
@@ -5004,7 +5007,7 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C7">
         <v>-1</v>
@@ -5015,7 +5018,7 @@
         <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C8">
         <v>-1</v>
@@ -5026,7 +5029,7 @@
         <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C9">
         <v>-1</v>
@@ -5037,7 +5040,7 @@
         <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C10">
         <v>-1</v>
@@ -5048,7 +5051,7 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C11">
         <v>-1</v>
@@ -5059,7 +5062,7 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C12">
         <v>-1</v>
@@ -5070,7 +5073,7 @@
         <v>18</v>
       </c>
       <c r="B13" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C13">
         <v>-1</v>
@@ -5081,7 +5084,7 @@
         <v>19</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C14">
         <v>-1</v>
@@ -5092,7 +5095,7 @@
         <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C15">
         <v>-1</v>
@@ -5103,7 +5106,7 @@
         <v>20</v>
       </c>
       <c r="B16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C16">
         <v>-1</v>
@@ -5114,7 +5117,7 @@
         <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C17">
         <v>-1</v>
@@ -5125,7 +5128,7 @@
         <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C18">
         <v>-1</v>
@@ -5136,7 +5139,7 @@
         <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C19">
         <v>-1</v>
@@ -5147,7 +5150,7 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C20">
         <v>-1</v>
@@ -5158,7 +5161,7 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C21">
         <v>-1</v>
@@ -5169,7 +5172,7 @@
         <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C22">
         <v>-1</v>
@@ -5180,7 +5183,7 @@
         <v>23</v>
       </c>
       <c r="B23" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C23">
         <v>-1</v>
@@ -5191,7 +5194,7 @@
         <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C24">
         <v>-1</v>
@@ -5202,7 +5205,7 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C25">
         <v>-1</v>
@@ -5213,7 +5216,7 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C26">
         <v>-1</v>
@@ -5224,7 +5227,7 @@
         <v>25</v>
       </c>
       <c r="B27" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C27">
         <v>-1</v>
@@ -5235,7 +5238,7 @@
         <v>26</v>
       </c>
       <c r="B28" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C28">
         <v>-1</v>
@@ -5246,7 +5249,7 @@
         <v>26</v>
       </c>
       <c r="B29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C29">
         <v>-1</v>
@@ -5257,7 +5260,7 @@
         <v>27</v>
       </c>
       <c r="B30" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C30">
         <v>-1</v>
@@ -5268,7 +5271,7 @@
         <v>27</v>
       </c>
       <c r="B31" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C31">
         <v>-1</v>
@@ -5279,7 +5282,7 @@
         <v>28</v>
       </c>
       <c r="B32" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C32">
         <v>-1</v>
@@ -5290,7 +5293,7 @@
         <v>28</v>
       </c>
       <c r="B33" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C33">
         <v>-1</v>
@@ -5301,7 +5304,7 @@
         <v>29</v>
       </c>
       <c r="B34" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C34">
         <v>-1</v>
@@ -5312,7 +5315,7 @@
         <v>29</v>
       </c>
       <c r="B35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C35">
         <v>-1</v>
@@ -5323,7 +5326,7 @@
         <v>30</v>
       </c>
       <c r="B36" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C36">
         <v>-1</v>
@@ -5334,7 +5337,7 @@
         <v>30</v>
       </c>
       <c r="B37" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C37">
         <v>-1</v>
@@ -5345,7 +5348,7 @@
         <v>31</v>
       </c>
       <c r="B38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C38">
         <v>-1</v>
@@ -5356,7 +5359,7 @@
         <v>31</v>
       </c>
       <c r="B39" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C39">
         <v>-1</v>
@@ -5367,7 +5370,7 @@
         <v>32</v>
       </c>
       <c r="B40" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C40">
         <v>-1</v>
@@ -5378,7 +5381,7 @@
         <v>32</v>
       </c>
       <c r="B41" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C41">
         <v>-1</v>
@@ -5389,7 +5392,7 @@
         <v>33</v>
       </c>
       <c r="B42" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C42">
         <v>-1</v>
@@ -5400,7 +5403,7 @@
         <v>33</v>
       </c>
       <c r="B43" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C43">
         <v>-1</v>
@@ -5411,7 +5414,7 @@
         <v>34</v>
       </c>
       <c r="B44" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C44">
         <v>-1</v>
@@ -5422,7 +5425,7 @@
         <v>34</v>
       </c>
       <c r="B45" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C45">
         <v>-1</v>
@@ -5433,7 +5436,7 @@
         <v>35</v>
       </c>
       <c r="B46" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C46">
         <v>-1</v>
@@ -5444,7 +5447,7 @@
         <v>35</v>
       </c>
       <c r="B47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C47">
         <v>-1</v>
@@ -5455,7 +5458,7 @@
         <v>36</v>
       </c>
       <c r="B48" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C48">
         <v>-1</v>
@@ -5466,7 +5469,7 @@
         <v>36</v>
       </c>
       <c r="B49" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C49">
         <v>-1</v>
@@ -5477,7 +5480,7 @@
         <v>37</v>
       </c>
       <c r="B50" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C50">
         <v>-1</v>
@@ -5488,7 +5491,7 @@
         <v>37</v>
       </c>
       <c r="B51" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C51">
         <v>-1</v>
@@ -5499,7 +5502,7 @@
         <v>38</v>
       </c>
       <c r="B52" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C52">
         <v>-1</v>
@@ -5510,7 +5513,7 @@
         <v>38</v>
       </c>
       <c r="B53" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C53">
         <v>-1</v>
@@ -5521,7 +5524,7 @@
         <v>39</v>
       </c>
       <c r="B54" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C54">
         <v>-1</v>
@@ -5532,7 +5535,7 @@
         <v>39</v>
       </c>
       <c r="B55" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C55">
         <v>-1</v>
@@ -5543,7 +5546,7 @@
         <v>40</v>
       </c>
       <c r="B56" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C56">
         <v>-1</v>
@@ -5554,7 +5557,7 @@
         <v>40</v>
       </c>
       <c r="B57" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C57">
         <v>-1</v>
@@ -5565,7 +5568,7 @@
         <v>41</v>
       </c>
       <c r="B58" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C58">
         <v>-1</v>
@@ -5576,7 +5579,7 @@
         <v>41</v>
       </c>
       <c r="B59" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C59">
         <v>-1</v>
@@ -5587,7 +5590,7 @@
         <v>42</v>
       </c>
       <c r="B60" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C60">
         <v>-1</v>
@@ -5598,7 +5601,7 @@
         <v>42</v>
       </c>
       <c r="B61" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C61">
         <v>-1</v>
@@ -5609,7 +5612,7 @@
         <v>43</v>
       </c>
       <c r="B62" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C62">
         <v>-1</v>
@@ -5620,7 +5623,7 @@
         <v>43</v>
       </c>
       <c r="B63" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C63">
         <v>-1</v>
@@ -5631,7 +5634,7 @@
         <v>44</v>
       </c>
       <c r="B64" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C64">
         <v>-1</v>
@@ -5642,7 +5645,7 @@
         <v>44</v>
       </c>
       <c r="B65" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C65">
         <v>-1</v>
@@ -5653,7 +5656,7 @@
         <v>45</v>
       </c>
       <c r="B66" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C66">
         <v>-1</v>
@@ -5664,7 +5667,7 @@
         <v>45</v>
       </c>
       <c r="B67" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C67">
         <v>-1</v>
@@ -5675,7 +5678,7 @@
         <v>46</v>
       </c>
       <c r="B68" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C68">
         <v>-1</v>
@@ -5686,7 +5689,7 @@
         <v>46</v>
       </c>
       <c r="B69" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C69">
         <v>-1</v>
@@ -5697,7 +5700,7 @@
         <v>47</v>
       </c>
       <c r="B70" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C70">
         <v>-1</v>
@@ -5708,7 +5711,7 @@
         <v>47</v>
       </c>
       <c r="B71" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C71">
         <v>-1</v>
@@ -5719,7 +5722,7 @@
         <v>48</v>
       </c>
       <c r="B72" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C72">
         <v>-1</v>
@@ -5730,7 +5733,7 @@
         <v>48</v>
       </c>
       <c r="B73" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C73">
         <v>-1</v>
@@ -5741,7 +5744,7 @@
         <v>49</v>
       </c>
       <c r="B74" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C74">
         <v>-1</v>
@@ -5752,7 +5755,7 @@
         <v>49</v>
       </c>
       <c r="B75" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C75">
         <v>-1</v>
@@ -5763,7 +5766,7 @@
         <v>50</v>
       </c>
       <c r="B76" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C76">
         <v>-1</v>
@@ -5774,7 +5777,7 @@
         <v>50</v>
       </c>
       <c r="B77" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C77">
         <v>-1</v>
@@ -5785,7 +5788,7 @@
         <v>51</v>
       </c>
       <c r="B78" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C78">
         <v>-1</v>
@@ -5796,7 +5799,7 @@
         <v>51</v>
       </c>
       <c r="B79" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C79">
         <v>-1</v>
@@ -5807,7 +5810,7 @@
         <v>52</v>
       </c>
       <c r="B80" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C80">
         <v>-1</v>
@@ -5818,7 +5821,7 @@
         <v>52</v>
       </c>
       <c r="B81" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C81">
         <v>-1</v>
@@ -5829,7 +5832,7 @@
         <v>53</v>
       </c>
       <c r="B82" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C82">
         <v>-1</v>
@@ -5840,7 +5843,7 @@
         <v>53</v>
       </c>
       <c r="B83" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C83">
         <v>-1</v>
@@ -5851,7 +5854,7 @@
         <v>54</v>
       </c>
       <c r="B84" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C84">
         <v>-1</v>
@@ -5862,7 +5865,7 @@
         <v>54</v>
       </c>
       <c r="B85" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C85">
         <v>-1</v>
@@ -5873,7 +5876,7 @@
         <v>55</v>
       </c>
       <c r="B86" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C86">
         <v>-1</v>
@@ -5884,7 +5887,7 @@
         <v>55</v>
       </c>
       <c r="B87" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C87">
         <v>-1</v>
@@ -5895,7 +5898,7 @@
         <v>56</v>
       </c>
       <c r="B88" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C88">
         <v>-1</v>
@@ -5906,7 +5909,7 @@
         <v>56</v>
       </c>
       <c r="B89" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C89">
         <v>-1</v>
@@ -5917,7 +5920,7 @@
         <v>57</v>
       </c>
       <c r="B90" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C90">
         <v>-1</v>
@@ -5928,7 +5931,7 @@
         <v>57</v>
       </c>
       <c r="B91" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C91">
         <v>-1</v>
@@ -5939,7 +5942,7 @@
         <v>58</v>
       </c>
       <c r="B92" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C92">
         <v>-1</v>
@@ -5950,7 +5953,7 @@
         <v>58</v>
       </c>
       <c r="B93" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C93">
         <v>-1</v>
@@ -5961,7 +5964,7 @@
         <v>59</v>
       </c>
       <c r="B94" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C94">
         <v>-1</v>
@@ -5972,7 +5975,7 @@
         <v>59</v>
       </c>
       <c r="B95" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C95">
         <v>-1</v>
@@ -5983,7 +5986,7 @@
         <v>60</v>
       </c>
       <c r="B96" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C96">
         <v>-1</v>
@@ -5994,7 +5997,7 @@
         <v>60</v>
       </c>
       <c r="B97" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C97">
         <v>-1</v>
@@ -6005,7 +6008,7 @@
         <v>61</v>
       </c>
       <c r="B98" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C98">
         <v>-1</v>
@@ -6016,7 +6019,7 @@
         <v>61</v>
       </c>
       <c r="B99" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C99">
         <v>-1</v>
@@ -6027,7 +6030,7 @@
         <v>62</v>
       </c>
       <c r="B100" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C100">
         <v>-1</v>
@@ -6038,7 +6041,7 @@
         <v>62</v>
       </c>
       <c r="B101" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C101">
         <v>-1</v>
@@ -6049,7 +6052,7 @@
         <v>63</v>
       </c>
       <c r="B102" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C102">
         <v>-1</v>
@@ -6060,7 +6063,7 @@
         <v>63</v>
       </c>
       <c r="B103" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C103">
         <v>-1</v>
@@ -6071,7 +6074,7 @@
         <v>64</v>
       </c>
       <c r="B104" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C104">
         <v>-1</v>
@@ -6082,7 +6085,7 @@
         <v>64</v>
       </c>
       <c r="B105" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C105">
         <v>-1</v>
@@ -6093,7 +6096,7 @@
         <v>65</v>
       </c>
       <c r="B106" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C106">
         <v>-1</v>
@@ -6104,7 +6107,7 @@
         <v>65</v>
       </c>
       <c r="B107" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C107">
         <v>-1</v>
@@ -6115,7 +6118,7 @@
         <v>66</v>
       </c>
       <c r="B108" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C108">
         <v>-1</v>
@@ -6126,7 +6129,7 @@
         <v>66</v>
       </c>
       <c r="B109" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C109">
         <v>-1</v>
@@ -6137,7 +6140,7 @@
         <v>67</v>
       </c>
       <c r="B110" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C110">
         <v>-1</v>
@@ -6148,7 +6151,7 @@
         <v>67</v>
       </c>
       <c r="B111" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C111">
         <v>-1</v>
@@ -6159,7 +6162,7 @@
         <v>68</v>
       </c>
       <c r="B112" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C112">
         <v>-1</v>
@@ -6170,7 +6173,7 @@
         <v>68</v>
       </c>
       <c r="B113" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C113">
         <v>-1</v>
@@ -6181,7 +6184,7 @@
         <v>69</v>
       </c>
       <c r="B114" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C114">
         <v>-1</v>
@@ -6192,7 +6195,7 @@
         <v>69</v>
       </c>
       <c r="B115" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C115">
         <v>-1</v>
@@ -6203,7 +6206,7 @@
         <v>70</v>
       </c>
       <c r="B116" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C116">
         <v>-1</v>
@@ -6214,7 +6217,7 @@
         <v>70</v>
       </c>
       <c r="B117" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C117">
         <v>-1</v>
@@ -6225,7 +6228,7 @@
         <v>71</v>
       </c>
       <c r="B118" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C118">
         <v>-1</v>
@@ -6236,7 +6239,7 @@
         <v>71</v>
       </c>
       <c r="B119" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C119">
         <v>-1</v>
@@ -6247,7 +6250,7 @@
         <v>72</v>
       </c>
       <c r="B120" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C120">
         <v>-1</v>
@@ -6258,7 +6261,7 @@
         <v>72</v>
       </c>
       <c r="B121" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C121">
         <v>-1</v>
@@ -6269,7 +6272,7 @@
         <v>73</v>
       </c>
       <c r="B122" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C122">
         <v>-1</v>
@@ -6280,7 +6283,7 @@
         <v>73</v>
       </c>
       <c r="B123" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C123">
         <v>-1</v>
@@ -6291,7 +6294,7 @@
         <v>74</v>
       </c>
       <c r="B124" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C124">
         <v>-1</v>
@@ -6302,7 +6305,7 @@
         <v>74</v>
       </c>
       <c r="B125" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C125">
         <v>-1</v>
@@ -6313,7 +6316,7 @@
         <v>75</v>
       </c>
       <c r="B126" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C126">
         <v>-1</v>
@@ -6324,7 +6327,7 @@
         <v>75</v>
       </c>
       <c r="B127" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C127">
         <v>-1</v>
@@ -6335,7 +6338,7 @@
         <v>76</v>
       </c>
       <c r="B128" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C128">
         <v>-1</v>
@@ -6346,7 +6349,7 @@
         <v>76</v>
       </c>
       <c r="B129" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C129">
         <v>-1</v>
@@ -6357,7 +6360,7 @@
         <v>77</v>
       </c>
       <c r="B130" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C130">
         <v>-1</v>
@@ -6368,7 +6371,7 @@
         <v>77</v>
       </c>
       <c r="B131" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C131">
         <v>-1</v>
@@ -6379,7 +6382,7 @@
         <v>78</v>
       </c>
       <c r="B132" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C132">
         <v>-1</v>
@@ -6390,7 +6393,7 @@
         <v>78</v>
       </c>
       <c r="B133" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C133">
         <v>-1</v>
@@ -6401,7 +6404,7 @@
         <v>79</v>
       </c>
       <c r="B134" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C134">
         <v>-1</v>
@@ -6412,7 +6415,7 @@
         <v>80</v>
       </c>
       <c r="B135" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C135">
         <v>-1</v>
@@ -6423,7 +6426,7 @@
         <v>80</v>
       </c>
       <c r="B136" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C136">
         <v>-1</v>
@@ -6434,7 +6437,7 @@
         <v>81</v>
       </c>
       <c r="B137" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C137">
         <v>-1</v>
@@ -6445,7 +6448,7 @@
         <v>81</v>
       </c>
       <c r="B138" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C138">
         <v>-1</v>
@@ -6456,7 +6459,7 @@
         <v>82</v>
       </c>
       <c r="B139" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C139">
         <v>-1</v>
@@ -6467,7 +6470,7 @@
         <v>82</v>
       </c>
       <c r="B140" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C140">
         <v>-1</v>
@@ -6478,7 +6481,7 @@
         <v>83</v>
       </c>
       <c r="B141" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C141">
         <v>-1</v>
@@ -6489,7 +6492,7 @@
         <v>83</v>
       </c>
       <c r="B142" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C142">
         <v>-1</v>
@@ -6500,7 +6503,7 @@
         <v>84</v>
       </c>
       <c r="B143" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C143">
         <v>-1</v>
@@ -6511,7 +6514,7 @@
         <v>84</v>
       </c>
       <c r="B144" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C144">
         <v>-1</v>
@@ -6522,7 +6525,7 @@
         <v>85</v>
       </c>
       <c r="B145" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C145">
         <v>-1</v>
@@ -6533,7 +6536,7 @@
         <v>85</v>
       </c>
       <c r="B146" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C146">
         <v>-1</v>
@@ -6544,7 +6547,7 @@
         <v>86</v>
       </c>
       <c r="B147" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C147">
         <v>-1</v>
@@ -6555,7 +6558,7 @@
         <v>86</v>
       </c>
       <c r="B148" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C148">
         <v>-1</v>
@@ -6566,7 +6569,7 @@
         <v>87</v>
       </c>
       <c r="B149" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C149">
         <v>-1</v>
@@ -6577,7 +6580,7 @@
         <v>87</v>
       </c>
       <c r="B150" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C150">
         <v>-1</v>
@@ -6588,7 +6591,7 @@
         <v>88</v>
       </c>
       <c r="B151" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C151">
         <v>-1</v>
@@ -6599,7 +6602,7 @@
         <v>88</v>
       </c>
       <c r="B152" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C152">
         <v>-1</v>
@@ -6610,7 +6613,7 @@
         <v>89</v>
       </c>
       <c r="B153" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C153">
         <v>-1</v>
@@ -6621,7 +6624,7 @@
         <v>89</v>
       </c>
       <c r="B154" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C154">
         <v>-1</v>
@@ -6632,7 +6635,7 @@
         <v>90</v>
       </c>
       <c r="B155" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C155">
         <v>-1</v>
@@ -6643,7 +6646,7 @@
         <v>90</v>
       </c>
       <c r="B156" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C156">
         <v>-1</v>
@@ -6654,7 +6657,7 @@
         <v>91</v>
       </c>
       <c r="B157" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C157">
         <v>-1</v>
@@ -6665,7 +6668,7 @@
         <v>91</v>
       </c>
       <c r="B158" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C158">
         <v>-1</v>
@@ -6683,7 +6686,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B1" t="s">
         <v>92</v>
@@ -6703,7 +6706,7 @@
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B2" t="s">
         <v>92</v>
@@ -6723,7 +6726,7 @@
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B3" t="s">
         <v>92</v>
@@ -6743,7 +6746,7 @@
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B4" t="s">
         <v>92</v>
@@ -6763,7 +6766,7 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B5" t="s">
         <v>92</v>
@@ -6783,7 +6786,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B6" t="s">
         <v>92</v>
@@ -6803,7 +6806,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B7" t="s">
         <v>92</v>
@@ -6823,7 +6826,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B8" t="s">
         <v>92</v>
@@ -6843,7 +6846,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B9" t="s">
         <v>92</v>
@@ -6863,7 +6866,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B10" t="s">
         <v>92</v>
@@ -6883,7 +6886,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B11" t="s">
         <v>92</v>
@@ -6903,7 +6906,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B12" t="s">
         <v>92</v>
@@ -6923,7 +6926,7 @@
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B13" t="s">
         <v>93</v>
@@ -6943,7 +6946,7 @@
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B14" t="s">
         <v>93</v>
@@ -6963,7 +6966,7 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B15" t="s">
         <v>93</v>
@@ -6983,7 +6986,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B16" t="s">
         <v>93</v>
@@ -7003,7 +7006,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="1" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B17" t="s">
         <v>93</v>
@@ -7023,7 +7026,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B18" t="s">
         <v>93</v>
@@ -7043,7 +7046,7 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B19" t="s">
         <v>93</v>
@@ -7063,7 +7066,7 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="1" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B20" t="s">
         <v>93</v>
@@ -7083,7 +7086,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="1" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B21" t="s">
         <v>93</v>
@@ -7103,7 +7106,7 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B22" t="s">
         <v>93</v>
@@ -7123,7 +7126,7 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B23" t="s">
         <v>93</v>
@@ -7143,7 +7146,7 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B24" t="s">
         <v>93</v>
@@ -7163,7 +7166,7 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B25" t="s">
         <v>94</v>
@@ -7183,7 +7186,7 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B26" t="s">
         <v>96</v>
@@ -7203,7 +7206,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B27" t="s">
         <v>96</v>
@@ -7223,7 +7226,7 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B28" t="s">
         <v>96</v>
@@ -7243,7 +7246,7 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B29" t="s">
         <v>96</v>
@@ -7263,7 +7266,7 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B30" t="s">
         <v>96</v>
@@ -7283,7 +7286,7 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="1" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B31" t="s">
         <v>95</v>
@@ -7303,7 +7306,7 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B32" t="s">
         <v>95</v>
@@ -7323,7 +7326,7 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B33" t="s">
         <v>95</v>
@@ -7343,7 +7346,7 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B34" t="s">
         <v>95</v>
@@ -7363,7 +7366,7 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B35" t="s">
         <v>95</v>
@@ -7383,7 +7386,7 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B36" t="s">
         <v>95</v>
@@ -7403,7 +7406,7 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B37" t="s">
         <v>95</v>
@@ -7423,7 +7426,7 @@
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="1" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B38" t="s">
         <v>95</v>
@@ -7443,7 +7446,7 @@
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B39" t="s">
         <v>95</v>
@@ -7463,7 +7466,7 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B40" t="s">
         <v>95</v>
@@ -7483,7 +7486,7 @@
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B41" t="s">
         <v>95</v>
@@ -7503,7 +7506,7 @@
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B42" t="s">
         <v>95</v>
@@ -7523,7 +7526,7 @@
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B43" t="s">
         <v>95</v>
@@ -7543,7 +7546,7 @@
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B44" t="s">
         <v>95</v>
@@ -7563,7 +7566,7 @@
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="1" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B45" t="s">
         <v>95</v>
@@ -7583,7 +7586,7 @@
     </row>
     <row r="46" spans="1:6">
       <c r="A46" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B46" t="s">
         <v>95</v>
@@ -7598,12 +7601,12 @@
         <v>99</v>
       </c>
       <c r="F46" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
     </row>
     <row r="47" spans="1:6">
       <c r="A47" s="1" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B47" t="s">
         <v>95</v>
@@ -7623,7 +7626,7 @@
     </row>
     <row r="48" spans="1:6">
       <c r="A48" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B48" t="s">
         <v>95</v>
@@ -7643,7 +7646,7 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B49" t="s">
         <v>95</v>
@@ -7663,7 +7666,7 @@
     </row>
     <row r="50" spans="1:6">
       <c r="A50" s="1" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B50" t="s">
         <v>95</v>
@@ -7683,7 +7686,7 @@
     </row>
     <row r="51" spans="1:6">
       <c r="A51" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B51" t="s">
         <v>95</v>
@@ -7703,7 +7706,7 @@
     </row>
     <row r="52" spans="1:6">
       <c r="A52" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B52" t="s">
         <v>95</v>
@@ -7723,7 +7726,7 @@
     </row>
     <row r="53" spans="1:6">
       <c r="A53" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B53" t="s">
         <v>95</v>
@@ -7743,7 +7746,7 @@
     </row>
     <row r="54" spans="1:6">
       <c r="A54" s="1" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B54" t="s">
         <v>95</v>
@@ -7758,12 +7761,12 @@
         <v>99</v>
       </c>
       <c r="F54" t="s">
-        <v>102</v>
+        <v>113</v>
       </c>
     </row>
     <row r="55" spans="1:6">
       <c r="A55" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B55" t="s">
         <v>95</v>
@@ -7783,7 +7786,7 @@
     </row>
     <row r="56" spans="1:6">
       <c r="A56" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B56" t="s">
         <v>95</v>
@@ -7803,7 +7806,7 @@
     </row>
     <row r="57" spans="1:6">
       <c r="A57" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B57" t="s">
         <v>95</v>

</xml_diff>